<commit_message>
Complete B residual analysis and update report handoff and task tracker
</commit_message>
<xml_diff>
--- a/reports/PHAN_CONG_2_NGUOI_IE313.xlsx
+++ b/reports/PHAN_CONG_2_NGUOI_IE313.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phân công" sheetId="1" r:id="Reac9eafd86214980"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lịch làm việc" sheetId="2" r:id="Re7c60a5a57b74bae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phân công" sheetId="1" r:id="R95fe3a6a73ed43ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lịch làm việc" sheetId="2" r:id="R16c0e2f63a684227"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -486,7 +486,7 @@
     <x:row r="5">
       <x:c r="A5" s="2"/>
       <x:c r="B5" s="4" t="str">
-        <x:v>Hoàn thành theo kiểm tra sản phẩm hiện có; không phải nghiệm thu giảng viên. A tiếp tục T08 sau nhận T07.</x:v>
+        <x:v>Hoàn thành theo kiểm tra sản phẩm hiện có; không phải nghiệm thu giảng viên. B đã hoàn tất T11; A tiếp tục T12/T14/T16 và sửa T03/T04.</x:v>
       </x:c>
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="2"/>
@@ -743,13 +743,13 @@
         <x:v>Cấu hình chung, xử lý đúng train/test, đóng băng test</x:v>
       </x:c>
       <x:c r="G15" s="15" t="str">
-        <x:v>Chờ kiểm tra</x:v>
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="H15" s="15" t="str">
-        <x:v>experiment_config.json; split_manifest.csv; experiment.py</x:v>
+        <x:v>experiment_config.json; split_manifest.csv; experiment.py; verify_a_t07.py; A_T07_ACCEPTANCE.md</x:v>
       </x:c>
       <x:c r="I15" s="15" t="str">
-        <x:v>Giao thức B đã kiểm 24 mục; A cần review và dùng đúng manifest/folds trước T08. Không chờ thêm B.</x:v>
+        <x:v>A đã kiểm toán 5 cổng (100% PASSED) và nghiệm thu chính thức; sẵn sàng làm T08.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" customHeight="1">
@@ -772,13 +772,13 @@
         <x:v>CV/train metrics; giải thích chọn biến, predictor không chứa target-derived bins</x:v>
       </x:c>
       <x:c r="G16" s="15" t="str">
-        <x:v>Chưa bắt đầu</x:v>
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="H16" s="15" t="str">
-        <x:v>HANDOFF_B_TO_A.md mục 4</x:v>
+        <x:v>Notebook 03a; a_models_cv_summary.csv; a_models_cv_folds.csv; fig_04; fig_05; A_T08_ACCEPTANCE.md</x:v>
       </x:c>
       <x:c r="I16" s="15" t="str">
-        <x:v>Chưa có output M0/M1/M2 từ A. A bắt đầu ngay với config/pipeline chung, chưa dùng test.</x:v>
+        <x:v>A đã hoàn thành 5-fold CV cho M0, M1, M2; trích xuất phương trình, hệ số; kiểm toán 5 cổng đạt 100% PASSED.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="84" customHeight="1">
@@ -830,13 +830,13 @@
         <x:v>Bảng MSE/RMSE/MAE/R², không dùng test để tune</x:v>
       </x:c>
       <x:c r="G18" s="15" t="str">
-        <x:v>Chưa bắt đầu</x:v>
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="H18" s="15" t="str">
-        <x:v>Chờ a_models_cv_summary.csv và T07</x:v>
+        <x:v>Notebook 04; model_comparison_cv_vs_test.csv; test_predictions.csv; fig_06; fig_07; A_B_T10_ACCEPTANCE.md</x:v>
       </x:c>
       <x:c r="I18" s="15" t="str">
-        <x:v>Chờ T08 của A; so CV chung, chốt mô hình rồi mới test cùng giao thức.</x:v>
+        <x:v>Chốt M3 chiến thắng trên CV; mở khóa đánh giá 10.342 mẫu test; kiểm toán 5 cổng đạt 100% PASSED.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -859,13 +859,13 @@
         <x:v>Notebook 04 và các hình thực tế, không gọi giá sai là gian lận</x:v>
       </x:c>
       <x:c r="G19" s="15" t="str">
-        <x:v>Chưa bắt đầu</x:v>
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="H19" s="15" t="str">
-        <x:v>Chờ test_predictions.csv từ T10</x:v>
+        <x:v>Notebook 05; b_residual_*; b_08–b_10; b_residual_verification.json</x:v>
       </x:c>
       <x:c r="I19" s="15" t="str">
-        <x:v>B cần actual/predicted + mã dòng test; không tạo residual giả hoặc dùng CV làm test.</x:v>
+        <x:v>Kernel mới 3 cell; 15 kiểm tra đạt. 1% mẫu chiếm 86,08% SSE; 167 dự đoán âm giữ nguyên. A dùng để tích hợp report/demo.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="84" customHeight="1">
@@ -920,10 +920,10 @@
         <x:v>Đang làm</x:v>
       </x:c>
       <x:c r="H21" s="15" t="str">
-        <x:v>eda_findings.md; b_model_findings.md</x:v>
+        <x:v>REPORT_B_SECTIONS.md; b_residual_findings.md; bảng CV/test thật</x:v>
       </x:c>
       <x:c r="I21" s="15" t="str">
-        <x:v>Đã có nội dung EDA/CV thật; chờ T08/T10 cho so sánh, test và kết luận cuối.</x:v>
+        <x:v>B hoàn tất nội dung EDA, CV, test, phần dư và kết luận. Chờ A tích hợp template Word/PDF và đọc chéo; không chờ B phân tích thêm.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -978,10 +978,10 @@
         <x:v>Đang làm</x:v>
       </x:c>
       <x:c r="H23" s="15" t="str">
-        <x:v>SLIDE_OUTLINE_B.md</x:v>
+        <x:v>SLIDE_OUTLINE_B.md cập nhật đủ T08/T10/T11 và lời nói B</x:v>
       </x:c>
       <x:c r="I23" s="15" t="str">
-        <x:v>Đã có dàn ý 13 slide/kịch bản; chưa có PPTX cuối, cần T08/T10 và thông tin nhóm.</x:v>
+        <x:v>B đã cập nhật nội dung/kịch bản kết quả. Chưa có PPTX cuối; còn thông tin nhóm, tích hợp, kiểm bố cục và diễn tập.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="84" customHeight="1">
@@ -1007,10 +1007,10 @@
         <x:v>Chưa bắt đầu</x:v>
       </x:c>
       <x:c r="H24" s="15" t="str">
-        <x:v>Chờ notebook cuối và demo</x:v>
+        <x:v>Notebook 01–05; NEXT_STEPS_A_20261013.md</x:v>
       </x:c>
       <x:c r="I24" s="15" t="str">
-        <x:v>A tích hợp và chạy sẵn; B có phần trình bày chuyên môn; chưa có demo cuối.</x:v>
+        <x:v>A tích hợp notebook cuối và chạy sạch; B đã có phần dư/kịch bản demo. Chưa hoàn tất demo cả nhóm.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="84" customHeight="1">
@@ -1093,7 +1093,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13d8b84135564eba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0e5a722fd5e4e3a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1219,7 +1219,7 @@
         <x:v>Khóa câu hỏi, schema và giao thức T07. Không loại hết biến chỉ vì r toàn bộ thấp</x:v>
       </x:c>
       <x:c r="E10" s="15" t="str">
-        <x:v>Chờ kiểm tra</x:v>
+        <x:v>Hoàn thành</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="66" customHeight="1">
@@ -1236,7 +1236,7 @@
         <x:v>Các mô hình lõi chạy được, CV trong train; không chọn theo test</x:v>
       </x:c>
       <x:c r="E11" s="15" t="str">
-        <x:v>Đang làm</x:v>
+        <x:v>Hoàn thành</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="66" customHeight="1">
@@ -1253,7 +1253,7 @@
         <x:v>Bảng kết quả cùng test/thang giá, mô hình chốt; báo thật kể cả R² thấp</x:v>
       </x:c>
       <x:c r="E12" s="15" t="str">
-        <x:v>Chưa bắt đầu</x:v>
+        <x:v>Hoàn thành</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="66" customHeight="1">
@@ -1339,7 +1339,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R593ec6710abc4ed8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra478ddca5b8048d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>